<commit_message>
Datos inspirados en distribuidora food service
- Productos con código AAA000 y categorías en mayúsculas (carnes, lácteos,
  abarrotes, conservas, congelados, etc.); 36 productos con imagen real
- Ventas con formato de comprobante FTxx-NNNNNNN
- 25 clientes: por vendedor, 2 de HOTELES Y ENTRETENIMIENTO, 2 de RESTAURANTES
  y 1 de rubro variado
- Pedidos nuevos generan id FT09-* coherente con el formato

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/clientes.xlsx
+++ b/data/clientes.xlsx
@@ -39,7 +39,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="006C4FD8"/>
+        <fgColor rgb="000D9488"/>
       </patternFill>
     </fill>
   </fills>
@@ -425,14 +425,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
@@ -482,22 +482,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bodega Don Pepe</t>
+          <t>Hotel Costa del Sol</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bodega</t>
+          <t>HOTELES Y ENTRETENIMIENTO</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tradicional</t>
+          <t>5 ESTRELLAS</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Esquina</t>
+          <t>CADENA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -519,22 +519,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Minimarket La Esquina</t>
+          <t>Hotel Sonesta Posadas</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Minimarket</t>
+          <t>HOTELES Y ENTRETENIMIENTO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Independiente</t>
+          <t>4 ESTRELLAS</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Barrio</t>
+          <t>CADENA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -556,22 +556,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Market Express SAC</t>
+          <t>Restaurante La Mar</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Minimarket</t>
+          <t>RESTAURANTES</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Cadena</t>
+          <t>MARINA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Centro</t>
+          <t>GOURMET</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -593,32 +593,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bodega Santa Rosa</t>
+          <t>Pollería Norkys</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Bodega</t>
+          <t>RESTAURANTES</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Tradicional</t>
+          <t>POLLERIA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Residencial</t>
+          <t>SALON</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>sofia@empresa.com</t>
+          <t>juan@empresa.com</t>
         </is>
       </c>
     </row>
@@ -630,32 +630,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Restaurante El Sabor</t>
+          <t>Panadería San Antonio</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>PANADERIAS Y PASTELERIAS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Menú</t>
+          <t>ARTESANAL</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Familiar</t>
+          <t>SALON</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>sofia@empresa.com</t>
+          <t>juan@empresa.com</t>
         </is>
       </c>
     </row>
@@ -667,22 +667,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Distribuidora Sur EIRL</t>
+          <t>Hotel Boutique Miraflores</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mayorista</t>
+          <t>HOTELES Y ENTRETENIMIENTO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Abarrotes</t>
+          <t>BOUTIQUE</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Zonal</t>
+          <t>INDEPENDIENTE</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -704,32 +704,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Bodega El Ahorro</t>
+          <t>Resort Las Dunas</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Bodega</t>
+          <t>HOTELES Y ENTRETENIMIENTO</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Tradicional</t>
+          <t>RESORT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Esquina</t>
+          <t>CADENA</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Arequipa</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>carlos@empresa.com</t>
+          <t>sofia@empresa.com</t>
         </is>
       </c>
     </row>
@@ -741,32 +741,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Minimarket Norteño</t>
+          <t>Cevichería El Muelle</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Minimarket</t>
+          <t>RESTAURANTES</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Independiente</t>
+          <t>CEVICHERIA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Avenida</t>
+          <t>MARINA</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Arequipa</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>carlos@empresa.com</t>
+          <t>sofia@empresa.com</t>
         </is>
       </c>
     </row>
@@ -778,32 +778,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bodega La Económica</t>
+          <t>Chifa Titi</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bodega</t>
+          <t>RESTAURANTES</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Tradicional</t>
+          <t>CHIFA</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Mercado</t>
+          <t>SALON</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Arequipa</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>ana@empresa.com</t>
+          <t>sofia@empresa.com</t>
         </is>
       </c>
     </row>
@@ -815,32 +815,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Pollería Brasa Roja</t>
+          <t>Cafetería Altomayo</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>CAFETERIAS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Pollería</t>
+          <t>ESPECIALIDAD</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Salón</t>
+          <t>CADENA</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Arequipa</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>ana@empresa.com</t>
+          <t>sofia@empresa.com</t>
         </is>
       </c>
     </row>
@@ -852,32 +852,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bodega Inka Wasi</t>
+          <t>Casino Atlantic City</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bodega</t>
+          <t>HOTELES Y ENTRETENIMIENTO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Tradicional</t>
+          <t>CASINO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Turístico</t>
+          <t>ENTRETENIMIENTO</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Piura</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>maria@empresa.com</t>
+          <t>carlos@empresa.com</t>
         </is>
       </c>
     </row>
@@ -889,30 +889,511 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Mayorista Andes SAC</t>
+          <t>Hotel La Hacienda</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mayorista</t>
+          <t>HOTELES Y ENTRETENIMIENTO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Abarrotes</t>
+          <t>4 ESTRELLAS</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Regional</t>
+          <t>INDEPENDIENTE</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>Piura</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>carlos@empresa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CL013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Parrillas El Tizón</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>RESTAURANTES</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>PARRILLA</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>GOURMET</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Piura</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>carlos@empresa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CL014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Restaurante Pardos</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>RESTAURANTES</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>POLLERIA</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CADENA</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Piura</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>carlos@empresa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CL015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Catering Eventos VIP</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CATERING Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CORPORATIVO</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>PREMIUM</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Piura</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>carlos@empresa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CL016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Casino Fiesta</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>HOTELES Y ENTRETENIMIENTO</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>CASINO</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Trujillo</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ana@empresa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CL017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Hotel Libertador</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>HOTELES Y ENTRETENIMIENTO</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>5 ESTRELLAS</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CADENA</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Trujillo</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>ana@empresa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CL018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Marisquería La Red</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>RESTAURANTES</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CEVICHERIA</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>MARINA</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Trujillo</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>ana@empresa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CL019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Restaurante El Aguajal</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>RESTAURANTES</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>CRIOLLO</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>FAMILIAR</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Trujillo</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>ana@empresa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CL020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Burger House Express</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>COMIDA RAPIDA</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>HAMBURGUESAS</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>FAST FOOD</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Trujillo</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>ana@empresa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CL021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Club Náutico Ancón</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>HOTELES Y ENTRETENIMIENTO</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>CLUB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>Cusco</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>maria@empresa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CL022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Hotel Plaza Real</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>HOTELES Y ENTRETENIMIENTO</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>BOUTIQUE</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Cusco</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>maria@empresa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CL023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Parrilla Don Carbón</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>RESTAURANTES</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>PARRILLA</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SALON</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Cusco</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>maria@empresa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CL024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Cevichería La Picantería</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>RESTAURANTES</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CEVICHERIA</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>FAMILIAR</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Cusco</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>maria@empresa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CL025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Minimarket La Canasta</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MINIMARKETS</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>BARRIO</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Cusco</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
         <is>
           <t>maria@empresa.com</t>
         </is>

</xml_diff>

<commit_message>
Todos los vendedores en la sede Lima
Los 5 vendedores y, por derivación, sus clientes quedan en sede Lima.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/clientes.xlsx
+++ b/data/clientes.xlsx
@@ -433,7 +433,7 @@
     <col width="29" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -687,7 +687,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -798,7 +798,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">

</xml_diff>

<commit_message>
Actualizar correo de Mario Gomez a mario@empresa.com
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/clientes.xlsx
+++ b/data/clientes.xlsx
@@ -1247,7 +1247,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>maria@empresa.com</t>
+          <t>mario@empresa.com</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>maria@empresa.com</t>
+          <t>mario@empresa.com</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>maria@empresa.com</t>
+          <t>mario@empresa.com</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>maria@empresa.com</t>
+          <t>mario@empresa.com</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>maria@empresa.com</t>
+          <t>mario@empresa.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Renombrar vendedores: Hugo Flores y Maria Gomez (con sus correos)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/clientes.xlsx
+++ b/data/clientes.xlsx
@@ -1062,7 +1062,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>ana@empresa.com</t>
+          <t>hugo@empresa.com</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>ana@empresa.com</t>
+          <t>hugo@empresa.com</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>ana@empresa.com</t>
+          <t>hugo@empresa.com</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>ana@empresa.com</t>
+          <t>hugo@empresa.com</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>ana@empresa.com</t>
+          <t>hugo@empresa.com</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>mario@empresa.com</t>
+          <t>maria@empresa.com</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>mario@empresa.com</t>
+          <t>maria@empresa.com</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>mario@empresa.com</t>
+          <t>maria@empresa.com</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>mario@empresa.com</t>
+          <t>maria@empresa.com</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>mario@empresa.com</t>
+          <t>maria@empresa.com</t>
         </is>
       </c>
     </row>

</xml_diff>